<commit_message>
feat(data): register ice cream machine input
- Add APP-019 as a one-unit candidate while keeping its location, model, and installation interfaces unknown until owner and vendor evidence arrives.

- Sync the equipment SSOT, workbook, PLUM/INT1/S-701 outputs, and route its 16 release blockers into one evidence request package.

- Validate workbook parity, 165/165 IFC scope, portable evidence hashes, and the reviewed-candidate release without changing the formal IFC.
</commit_message>
<xml_diff>
--- a/output/forms/滨海湾施工输入清单.xlsx
+++ b/output/forms/滨海湾施工输入清单.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R12f6e77aaf654ff0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="设计决策" sheetId="2" r:id="Rb53443d410f34dc8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="家电清单" sheetId="3" r:id="R0c1766789ce24516"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="设备主表" sheetId="4" r:id="R47205748a0bf472c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="安装条件" sheetId="5" r:id="R5f3e027b68514eb4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="证据索引" sheetId="6" r:id="R9bfd93135eaa4151"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R4c5883d2fa1a4283"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="设计决策" sheetId="2" r:id="R0810f7986ab34c9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="家电清单" sheetId="3" r:id="Rc94fa4b790144a05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="设备主表" sheetId="4" r:id="R17647ea015f94f4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="安装条件" sheetId="5" r:id="R69b02d8dac37430b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="证据索引" sheetId="6" r:id="R65f0e6b9615d4a6a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2782,9 +2782,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3e106c8b5fe45a2"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc999c6bcdfe14a1c"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra77a463d18d54dc8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0dd89f17ea04ed3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3815,6 +3815,44 @@
         <x:v>实际箱内运行已确认；补底部铭牌与设备功能</x:v>
       </x:c>
     </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>APP-019</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>冰淇淋机</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>甜品设备</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>待确认位置</x:v>
+      </x:c>
+      <x:c r="E20" t="str">
+        <x:v>待确认位置</x:v>
+      </x:c>
+      <x:c r="F20" t="str"/>
+      <x:c r="G20" t="str"/>
+      <x:c r="H20" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I20" t="str"/>
+      <x:c r="J20" t="str"/>
+      <x:c r="K20" t="str"/>
+      <x:c r="L20" t="str"/>
+      <x:c r="M20" t="str"/>
+      <x:c r="N20" t="str"/>
+      <x:c r="O20" t="str"/>
+      <x:c r="P20" t="str">
+        <x:v>业主确认新增一台冰淇淋机；未提供品牌、型号、位置或安装资料</x:v>
+      </x:c>
+      <x:c r="Q20" t="str">
+        <x:v>部分确认</x:v>
+      </x:c>
+      <x:c r="R20" t="str">
+        <x:v>候选设备，非已选/已购；不计入 NS-01/NS-02 负荷，待位置和准确型号后再决定插座、回路与给排水。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="Q2:Q19">
     <x:cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="已确认"/>
@@ -3839,7 +3877,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5990f0cd9f2f44c9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fd00120646e467f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15592,13 +15630,81 @@
         <x:v>APP-017 叠放套装的上部独立设备；产品尺寸不是接口中心。</x:v>
       </x:c>
     </x:row>
+    <x:row r="164">
+      <x:c r="A164" t="str">
+        <x:v>APP-019</x:v>
+      </x:c>
+      <x:c r="B164" t="str">
+        <x:v>APPLIANCE</x:v>
+      </x:c>
+      <x:c r="C164" t="str">
+        <x:v>甜品设备</x:v>
+      </x:c>
+      <x:c r="D164" t="str">
+        <x:v>冰淇淋机</x:v>
+      </x:c>
+      <x:c r="E164" t="str"/>
+      <x:c r="F164" t="str"/>
+      <x:c r="G164" t="str"/>
+      <x:c r="H164" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I164" t="str">
+        <x:v>candidate</x:v>
+      </x:c>
+      <x:c r="J164" t="str">
+        <x:v>partial</x:v>
+      </x:c>
+      <x:c r="K164" t="str">
+        <x:v>待确认位置</x:v>
+      </x:c>
+      <x:c r="L164" t="str">
+        <x:v>待确认位置</x:v>
+      </x:c>
+      <x:c r="M164" t="str"/>
+      <x:c r="N164" t="str"/>
+      <x:c r="O164" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="P164" t="str">
+        <x:v>logical_input</x:v>
+      </x:c>
+      <x:c r="Q164" t="str">
+        <x:v>APP-019</x:v>
+      </x:c>
+      <x:c r="R164" t="str"/>
+      <x:c r="S164" t="str"/>
+      <x:c r="T164" t="str"/>
+      <x:c r="U164" t="str"/>
+      <x:c r="V164" t="str">
+        <x:v>OWNER-INPUT-APP019-20260815</x:v>
+      </x:c>
+      <x:c r="W164" t="str">
+        <x:v>业主确认新增一台冰淇淋机；未提供品牌、型号、位置或安装资料</x:v>
+      </x:c>
+      <x:c r="X164" t="str">
+        <x:v>1.00</x:v>
+      </x:c>
+      <x:c r="Y164" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="Z164" t="str">
+        <x:v>appliance</x:v>
+      </x:c>
+      <x:c r="AA164" t="str">
+        <x:v>APP-019</x:v>
+      </x:c>
+      <x:c r="AB164" t="str">
+        <x:v>候选设备，非已选/已购；不计入 NS-01/NS-02 负荷，待位置和准确型号后再决定插座、回路与给排水。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:AB1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c8ac1a5c68c405c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbfc7efc78db4e2b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -44986,132 +45092,616 @@
       </x:c>
     </x:row>
     <x:row r="821" ht="31.5" customHeight="1">
-      <x:c r="A821" s="189"/>
-      <x:c r="B821" s="189"/>
-      <x:c r="C821" s="189"/>
-      <x:c r="D821" s="189"/>
-      <x:c r="E821" s="189"/>
-      <x:c r="F821" s="189"/>
-      <x:c r="G821" s="189"/>
-      <x:c r="H821" s="189"/>
-      <x:c r="I821" s="189"/>
-      <x:c r="J821" s="189"/>
-      <x:c r="K821" s="189"/>
-      <x:c r="L821" s="189"/>
-      <x:c r="M821" s="189"/>
-      <x:c r="N821" s="189"/>
+      <x:c r="A821" s="189" t="str">
+        <x:v>REQ-APP019-001</x:v>
+      </x:c>
+      <x:c r="B821" s="189" t="str">
+        <x:v>APP-019</x:v>
+      </x:c>
+      <x:c r="C821" s="189" t="str">
+        <x:v>ELEC</x:v>
+      </x:c>
+      <x:c r="D821" s="189" t="str">
+        <x:v>rated_power</x:v>
+      </x:c>
+      <x:c r="E821" s="189" t="str"/>
+      <x:c r="F821" s="189" t="str"/>
+      <x:c r="G821" s="189" t="str">
+        <x:v>W</x:v>
+      </x:c>
+      <x:c r="H821" s="189" t="str"/>
+      <x:c r="I821" s="189" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="J821" s="189" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="K821" s="189" t="str">
+        <x:v>OWNER-INPUT-APP019-20260815</x:v>
+      </x:c>
+      <x:c r="L821" s="189" t="str">
+        <x:v>业主仅确认设备类别与数量</x:v>
+      </x:c>
+      <x:c r="M821" s="189" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="N821" s="189" t="str">
+        <x:v>保持 unknown；关闭证据：准确型号名牌功率。</x:v>
+      </x:c>
     </x:row>
     <x:row r="822" ht="31.5" customHeight="1">
-      <x:c r="A822" s="189"/>
-      <x:c r="B822" s="189"/>
-      <x:c r="C822" s="189"/>
-      <x:c r="D822" s="189"/>
-      <x:c r="E822" s="189"/>
-      <x:c r="F822" s="189"/>
-      <x:c r="G822" s="189"/>
-      <x:c r="H822" s="189"/>
-      <x:c r="I822" s="189"/>
-      <x:c r="J822" s="189"/>
-      <x:c r="K822" s="189"/>
-      <x:c r="L822" s="189"/>
-      <x:c r="M822" s="189"/>
-      <x:c r="N822" s="189"/>
+      <x:c r="A822" s="189" t="str">
+        <x:v>REQ-APP019-002</x:v>
+      </x:c>
+      <x:c r="B822" s="189" t="str">
+        <x:v>APP-019</x:v>
+      </x:c>
+      <x:c r="C822" s="189" t="str">
+        <x:v>ELEC</x:v>
+      </x:c>
+      <x:c r="D822" s="189" t="str">
+        <x:v>simultaneous_group</x:v>
+      </x:c>
+      <x:c r="E822" s="189" t="str"/>
+      <x:c r="F822" s="189" t="str"/>
+      <x:c r="G822" s="189" t="str"/>
+      <x:c r="H822" s="189" t="str"/>
+      <x:c r="I822" s="189" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="J822" s="189" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="K822" s="189" t="str">
+        <x:v>OWNER-INPUT-APP019-20260815</x:v>
+      </x:c>
+      <x:c r="L822" s="189" t="str">
+        <x:v>业主仅确认设备类别与数量</x:v>
+      </x:c>
+      <x:c r="M822" s="189" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="N822" s="189" t="str">
+        <x:v>保持 unknown；关闭证据：使用位置和同时工况。</x:v>
+      </x:c>
     </x:row>
     <x:row r="823" ht="31.5" customHeight="1">
-      <x:c r="A823" s="189"/>
-      <x:c r="B823" s="189"/>
-      <x:c r="C823" s="189"/>
-      <x:c r="D823" s="189"/>
-      <x:c r="E823" s="189"/>
-      <x:c r="F823" s="189"/>
-      <x:c r="G823" s="189"/>
-      <x:c r="H823" s="189"/>
-      <x:c r="I823" s="189"/>
-      <x:c r="J823" s="189"/>
-      <x:c r="K823" s="189"/>
-      <x:c r="L823" s="189"/>
-      <x:c r="M823" s="189"/>
-      <x:c r="N823" s="189"/>
+      <x:c r="A823" s="189" t="str">
+        <x:v>REQ-APP019-003</x:v>
+      </x:c>
+      <x:c r="B823" s="189" t="str">
+        <x:v>APP-019</x:v>
+      </x:c>
+      <x:c r="C823" s="189" t="str">
+        <x:v>PLUM</x:v>
+      </x:c>
+      <x:c r="D823" s="189" t="str">
+        <x:v>water_required</x:v>
+      </x:c>
+      <x:c r="E823" s="189" t="str"/>
+      <x:c r="F823" s="189" t="str"/>
+      <x:c r="G823" s="189" t="str"/>
+      <x:c r="H823" s="189" t="str"/>
+      <x:c r="I823" s="189" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="J823" s="189" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="K823" s="189" t="str">
+        <x:v>OWNER-INPUT-APP019-20260815</x:v>
+      </x:c>
+      <x:c r="L823" s="189" t="str">
+        <x:v>业主仅确认设备类别与数量</x:v>
+      </x:c>
+      <x:c r="M823" s="189" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="N823" s="189" t="str">
+        <x:v>保持 unknown；关闭证据：准确型号安装图。</x:v>
+      </x:c>
     </x:row>
     <x:row r="824" ht="31.5" customHeight="1">
-      <x:c r="A824" s="189"/>
-      <x:c r="B824" s="189"/>
-      <x:c r="C824" s="189"/>
-      <x:c r="D824" s="189"/>
-      <x:c r="E824" s="189"/>
-      <x:c r="F824" s="189"/>
-      <x:c r="G824" s="189"/>
-      <x:c r="H824" s="189"/>
-      <x:c r="I824" s="189"/>
-      <x:c r="J824" s="189"/>
-      <x:c r="K824" s="189"/>
-      <x:c r="L824" s="189"/>
-      <x:c r="M824" s="189"/>
-      <x:c r="N824" s="189"/>
+      <x:c r="A824" s="189" t="str">
+        <x:v>REQ-APP019-004</x:v>
+      </x:c>
+      <x:c r="B824" s="189" t="str">
+        <x:v>APP-019</x:v>
+      </x:c>
+      <x:c r="C824" s="189" t="str">
+        <x:v>PLUM</x:v>
+      </x:c>
+      <x:c r="D824" s="189" t="str">
+        <x:v>drain_required</x:v>
+      </x:c>
+      <x:c r="E824" s="189" t="str"/>
+      <x:c r="F824" s="189" t="str"/>
+      <x:c r="G824" s="189" t="str"/>
+      <x:c r="H824" s="189" t="str"/>
+      <x:c r="I824" s="189" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="J824" s="189" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="K824" s="189" t="str">
+        <x:v>OWNER-INPUT-APP019-20260815</x:v>
+      </x:c>
+      <x:c r="L824" s="189" t="str">
+        <x:v>业主仅确认设备类别与数量</x:v>
+      </x:c>
+      <x:c r="M824" s="189" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="N824" s="189" t="str">
+        <x:v>保持 unknown；关闭证据：准确型号安装图。</x:v>
+      </x:c>
     </x:row>
     <x:row r="825" ht="31.5" customHeight="1">
-      <x:c r="A825" s="189"/>
-      <x:c r="B825" s="189"/>
-      <x:c r="C825" s="189"/>
-      <x:c r="D825" s="189"/>
-      <x:c r="E825" s="189"/>
-      <x:c r="F825" s="189"/>
-      <x:c r="G825" s="189"/>
-      <x:c r="H825" s="189"/>
-      <x:c r="I825" s="189"/>
-      <x:c r="J825" s="189"/>
-      <x:c r="K825" s="189"/>
-      <x:c r="L825" s="189"/>
-      <x:c r="M825" s="189"/>
-      <x:c r="N825" s="189"/>
+      <x:c r="A825" s="189" t="str">
+        <x:v>REQ-APP019-005</x:v>
+      </x:c>
+      <x:c r="B825" s="189" t="str">
+        <x:v>APP-019</x:v>
+      </x:c>
+      <x:c r="C825" s="189" t="str">
+        <x:v>GAS</x:v>
+      </x:c>
+      <x:c r="D825" s="189" t="str">
+        <x:v>gas_required</x:v>
+      </x:c>
+      <x:c r="E825" s="189" t="str"/>
+      <x:c r="F825" s="189" t="str"/>
+      <x:c r="G825" s="189" t="str"/>
+      <x:c r="H825" s="189" t="str"/>
+      <x:c r="I825" s="189" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="J825" s="189" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="K825" s="189" t="str">
+        <x:v>OWNER-INPUT-APP019-20260815</x:v>
+      </x:c>
+      <x:c r="L825" s="189" t="str">
+        <x:v>业主仅确认设备类别与数量</x:v>
+      </x:c>
+      <x:c r="M825" s="189" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="N825" s="189" t="str">
+        <x:v>保持 unknown；关闭证据：准确型号安装图。</x:v>
+      </x:c>
     </x:row>
     <x:row r="826" ht="31.5" customHeight="1">
-      <x:c r="A826" s="189"/>
-      <x:c r="B826" s="189"/>
-      <x:c r="C826" s="189"/>
-      <x:c r="D826" s="189"/>
-      <x:c r="E826" s="189"/>
-      <x:c r="F826" s="189"/>
-      <x:c r="G826" s="189"/>
-      <x:c r="H826" s="189"/>
-      <x:c r="I826" s="189"/>
-      <x:c r="J826" s="189"/>
-      <x:c r="K826" s="189"/>
-      <x:c r="L826" s="189"/>
-      <x:c r="M826" s="189"/>
-      <x:c r="N826" s="189"/>
+      <x:c r="A826" s="189" t="str">
+        <x:v>REQ-APP019-006</x:v>
+      </x:c>
+      <x:c r="B826" s="189" t="str">
+        <x:v>APP-019</x:v>
+      </x:c>
+      <x:c r="C826" s="189" t="str">
+        <x:v>HVAC/INT1</x:v>
+      </x:c>
+      <x:c r="D826" s="189" t="str">
+        <x:v>ventilation_required</x:v>
+      </x:c>
+      <x:c r="E826" s="189" t="str"/>
+      <x:c r="F826" s="189" t="str"/>
+      <x:c r="G826" s="189" t="str"/>
+      <x:c r="H826" s="189" t="str"/>
+      <x:c r="I826" s="189" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="J826" s="189" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="K826" s="189" t="str">
+        <x:v>OWNER-INPUT-APP019-20260815</x:v>
+      </x:c>
+      <x:c r="L826" s="189" t="str">
+        <x:v>业主仅确认设备类别与数量</x:v>
+      </x:c>
+      <x:c r="M826" s="189" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="N826" s="189" t="str">
+        <x:v>保持 unknown；关闭证据：准确型号散热和净距要求。</x:v>
+      </x:c>
     </x:row>
     <x:row r="827" ht="31.5" customHeight="1">
-      <x:c r="A827" s="189"/>
-      <x:c r="B827" s="189"/>
-      <x:c r="C827" s="189"/>
-      <x:c r="D827" s="189"/>
-      <x:c r="E827" s="189"/>
-      <x:c r="F827" s="189"/>
-      <x:c r="G827" s="189"/>
-      <x:c r="H827" s="189"/>
-      <x:c r="I827" s="189"/>
-      <x:c r="J827" s="189"/>
-      <x:c r="K827" s="189"/>
-      <x:c r="L827" s="189"/>
-      <x:c r="M827" s="189"/>
-      <x:c r="N827" s="189"/>
+      <x:c r="A827" s="189" t="str">
+        <x:v>REQ-APP019-007</x:v>
+      </x:c>
+      <x:c r="B827" s="189" t="str">
+        <x:v>APP-019</x:v>
+      </x:c>
+      <x:c r="C827" s="189" t="str">
+        <x:v>INT1</x:v>
+      </x:c>
+      <x:c r="D827" s="189" t="str">
+        <x:v>installation_mode</x:v>
+      </x:c>
+      <x:c r="E827" s="189" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="F827" s="189" t="str"/>
+      <x:c r="G827" s="189" t="str"/>
+      <x:c r="H827" s="189" t="str"/>
+      <x:c r="I827" s="189" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="J827" s="189" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="K827" s="189" t="str">
+        <x:v>OWNER-INPUT-APP019-20260815</x:v>
+      </x:c>
+      <x:c r="L827" s="189" t="str">
+        <x:v>业主仅确认设备类别与数量</x:v>
+      </x:c>
+      <x:c r="M827" s="189" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="N827" s="189" t="str">
+        <x:v>保持 unknown；关闭证据：台面、落地或嵌入形式。</x:v>
+      </x:c>
     </x:row>
     <x:row r="828" ht="31.5" customHeight="1">
-      <x:c r="A828" s="189"/>
-      <x:c r="B828" s="189"/>
-      <x:c r="C828" s="189"/>
-      <x:c r="D828" s="189"/>
-      <x:c r="E828" s="189"/>
-      <x:c r="F828" s="189"/>
-      <x:c r="G828" s="189"/>
-      <x:c r="H828" s="189"/>
-      <x:c r="I828" s="189"/>
-      <x:c r="J828" s="189"/>
-      <x:c r="K828" s="189"/>
-      <x:c r="L828" s="189"/>
-      <x:c r="M828" s="189"/>
-      <x:c r="N828" s="189"/>
+      <x:c r="A828" s="189" t="str">
+        <x:v>REQ-APP019-008</x:v>
+      </x:c>
+      <x:c r="B828" s="189" t="str">
+        <x:v>APP-019</x:v>
+      </x:c>
+      <x:c r="C828" s="189" t="str">
+        <x:v>ELEC</x:v>
+      </x:c>
+      <x:c r="D828" s="189" t="str">
+        <x:v>appliance_plug_rating_a</x:v>
+      </x:c>
+      <x:c r="E828" s="189" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="F828" s="189" t="str"/>
+      <x:c r="G828" s="189" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H828" s="189" t="str"/>
+      <x:c r="I828" s="189" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="J828" s="189" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="K828" s="189" t="str">
+        <x:v>OWNER-INPUT-APP019-20260815</x:v>
+      </x:c>
+      <x:c r="L828" s="189" t="str">
+        <x:v>业主仅确认设备类别与数量</x:v>
+      </x:c>
+      <x:c r="M828" s="189" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="N828" s="189" t="str">
+        <x:v>保持 unknown；关闭证据：实物插头或厂家电气页。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="829">
+      <x:c r="A829" t="str">
+        <x:v>REQ-APP019-009</x:v>
+      </x:c>
+      <x:c r="B829" t="str">
+        <x:v>APP-019</x:v>
+      </x:c>
+      <x:c r="C829" t="str">
+        <x:v>ELEC</x:v>
+      </x:c>
+      <x:c r="D829" t="str">
+        <x:v>wall_socket_rating_a</x:v>
+      </x:c>
+      <x:c r="E829" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="F829" t="str"/>
+      <x:c r="G829" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H829" t="str"/>
+      <x:c r="I829" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="J829" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="K829" t="str">
+        <x:v>OWNER-INPUT-APP019-20260815</x:v>
+      </x:c>
+      <x:c r="L829" t="str">
+        <x:v>业主仅确认设备类别与数量</x:v>
+      </x:c>
+      <x:c r="M829" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="N829" t="str">
+        <x:v>保持 unknown；关闭证据：按实购插头和支路计算匹配。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="830">
+      <x:c r="A830" t="str">
+        <x:v>REQ-APP019-010</x:v>
+      </x:c>
+      <x:c r="B830" t="str">
+        <x:v>APP-019</x:v>
+      </x:c>
+      <x:c r="C830" t="str">
+        <x:v>ELEC</x:v>
+      </x:c>
+      <x:c r="D830" t="str">
+        <x:v>branch_breaker_rating_a</x:v>
+      </x:c>
+      <x:c r="E830" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="F830" t="str"/>
+      <x:c r="G830" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H830" t="str"/>
+      <x:c r="I830" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="J830" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="K830" t="str">
+        <x:v>OWNER-INPUT-APP019-20260815</x:v>
+      </x:c>
+      <x:c r="L830" t="str">
+        <x:v>业主仅确认设备类别与数量</x:v>
+      </x:c>
+      <x:c r="M830" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="N830" t="str">
+        <x:v>保持 unknown；关闭证据：名牌负荷、同时工况和回路计算。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="831">
+      <x:c r="A831" t="str">
+        <x:v>REQ-APP019-011</x:v>
+      </x:c>
+      <x:c r="B831" t="str">
+        <x:v>APP-019</x:v>
+      </x:c>
+      <x:c r="C831" t="str">
+        <x:v>ELEC</x:v>
+      </x:c>
+      <x:c r="D831" t="str">
+        <x:v>dedicated_branch_circuit</x:v>
+      </x:c>
+      <x:c r="E831" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="F831" t="str"/>
+      <x:c r="G831" t="str"/>
+      <x:c r="H831" t="str"/>
+      <x:c r="I831" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="J831" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="K831" t="str">
+        <x:v>OWNER-INPUT-APP019-20260815</x:v>
+      </x:c>
+      <x:c r="L831" t="str">
+        <x:v>业主仅确认设备类别与数量</x:v>
+      </x:c>
+      <x:c r="M831" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="N831" t="str">
+        <x:v>保持 unknown；关闭证据：名牌负荷、位置和共路工况。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="832">
+      <x:c r="A832" t="str">
+        <x:v>REQ-APP019-012</x:v>
+      </x:c>
+      <x:c r="B832" t="str">
+        <x:v>APP-019</x:v>
+      </x:c>
+      <x:c r="C832" t="str">
+        <x:v>INT1</x:v>
+      </x:c>
+      <x:c r="D832" t="str">
+        <x:v>product_width</x:v>
+      </x:c>
+      <x:c r="E832" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="F832" t="str"/>
+      <x:c r="G832" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="H832" t="str"/>
+      <x:c r="I832" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="J832" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="K832" t="str">
+        <x:v>OWNER-INPUT-APP019-20260815</x:v>
+      </x:c>
+      <x:c r="L832" t="str">
+        <x:v>业主仅确认设备类别与数量</x:v>
+      </x:c>
+      <x:c r="M832" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="N832" t="str">
+        <x:v>保持 unknown；关闭证据：准确型号尺寸图。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="833">
+      <x:c r="A833" t="str">
+        <x:v>REQ-APP019-013</x:v>
+      </x:c>
+      <x:c r="B833" t="str">
+        <x:v>APP-019</x:v>
+      </x:c>
+      <x:c r="C833" t="str">
+        <x:v>INT1</x:v>
+      </x:c>
+      <x:c r="D833" t="str">
+        <x:v>product_height</x:v>
+      </x:c>
+      <x:c r="E833" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="F833" t="str"/>
+      <x:c r="G833" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="H833" t="str"/>
+      <x:c r="I833" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="J833" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="K833" t="str">
+        <x:v>OWNER-INPUT-APP019-20260815</x:v>
+      </x:c>
+      <x:c r="L833" t="str">
+        <x:v>业主仅确认设备类别与数量</x:v>
+      </x:c>
+      <x:c r="M833" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="N833" t="str">
+        <x:v>保持 unknown；关闭证据：准确型号尺寸图。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="834">
+      <x:c r="A834" t="str">
+        <x:v>REQ-APP019-014</x:v>
+      </x:c>
+      <x:c r="B834" t="str">
+        <x:v>APP-019</x:v>
+      </x:c>
+      <x:c r="C834" t="str">
+        <x:v>INT1</x:v>
+      </x:c>
+      <x:c r="D834" t="str">
+        <x:v>product_depth</x:v>
+      </x:c>
+      <x:c r="E834" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="F834" t="str"/>
+      <x:c r="G834" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="H834" t="str"/>
+      <x:c r="I834" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="J834" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="K834" t="str">
+        <x:v>OWNER-INPUT-APP019-20260815</x:v>
+      </x:c>
+      <x:c r="L834" t="str">
+        <x:v>业主仅确认设备类别与数量</x:v>
+      </x:c>
+      <x:c r="M834" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="N834" t="str">
+        <x:v>保持 unknown；关闭证据：准确型号尺寸图。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="835">
+      <x:c r="A835" t="str">
+        <x:v>REQ-APP019-015</x:v>
+      </x:c>
+      <x:c r="B835" t="str">
+        <x:v>APP-019</x:v>
+      </x:c>
+      <x:c r="C835" t="str">
+        <x:v>INT1</x:v>
+      </x:c>
+      <x:c r="D835" t="str">
+        <x:v>service_clearance</x:v>
+      </x:c>
+      <x:c r="E835" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="F835" t="str"/>
+      <x:c r="G835" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="H835" t="str"/>
+      <x:c r="I835" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="J835" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="K835" t="str">
+        <x:v>OWNER-INPUT-APP019-20260815</x:v>
+      </x:c>
+      <x:c r="L835" t="str">
+        <x:v>业主仅确认设备类别与数量</x:v>
+      </x:c>
+      <x:c r="M835" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="N835" t="str">
+        <x:v>保持 unknown；关闭证据：厂家散热、操作和检修要求。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="836">
+      <x:c r="A836" t="str">
+        <x:v>REQ-APP019-016</x:v>
+      </x:c>
+      <x:c r="B836" t="str">
+        <x:v>APP-019</x:v>
+      </x:c>
+      <x:c r="C836" t="str">
+        <x:v>MULTI</x:v>
+      </x:c>
+      <x:c r="D836" t="str">
+        <x:v>interface_center_coordinates</x:v>
+      </x:c>
+      <x:c r="E836" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="F836" t="str"/>
+      <x:c r="G836" t="str"/>
+      <x:c r="H836" t="str"/>
+      <x:c r="I836" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="J836" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="K836" t="str">
+        <x:v>OWNER-INPUT-APP019-20260815</x:v>
+      </x:c>
+      <x:c r="L836" t="str">
+        <x:v>业主仅确认设备类别与数量</x:v>
+      </x:c>
+      <x:c r="M836" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="N836" t="str">
+        <x:v>保持 unknown；关闭证据：厂家安装图与项目定位。</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -45119,7 +45709,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ab72e9b49f74bfa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3762d03ab23049c3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -57020,13 +57610,77 @@
         <x:v>请求包只定义最短关闭证据，不把待回复字段标为已确认。</x:v>
       </x:c>
     </x:row>
+    <x:row r="183">
+      <x:c r="A183" t="str">
+        <x:v>OWNER-INPUT-APP019-20260815</x:v>
+      </x:c>
+      <x:c r="B183" t="str">
+        <x:v>ELEC/PLUM/INT1</x:v>
+      </x:c>
+      <x:c r="C183" t="str">
+        <x:v>E-303/P-201/P-202/INT1/S-701</x:v>
+      </x:c>
+      <x:c r="D183" t="str">
+        <x:v>APP-019 冰淇淋机设备类别与数量</x:v>
+      </x:c>
+      <x:c r="E183" t="str">
+        <x:v>owner_confirmation</x:v>
+      </x:c>
+      <x:c r="F183" t="str">
+        <x:v>drawings/evidence/OWNER-INPUT-APP-019-20260815.md</x:v>
+      </x:c>
+      <x:c r="G183" t="str"/>
+      <x:c r="H183" t="str">
+        <x:v>drawings/evidence/OWNER-INPUT-APP-019-20260815.md</x:v>
+      </x:c>
+      <x:c r="I183" t="str">
+        <x:v>0004eeccf0a7f076485a2bf5d663df6e7ab26cf696398639728d8fbb5e4d614c</x:v>
+      </x:c>
+      <x:c r="J183" t="str">
+        <x:v>业主新增一台冰淇淋机</x:v>
+      </x:c>
+      <x:c r="K183" t="str">
+        <x:v>业主确认新增冰淇淋机 1 台</x:v>
+      </x:c>
+      <x:c r="L183" t="str">
+        <x:v>项目需要登记一台冰淇淋机</x:v>
+      </x:c>
+      <x:c r="M183" t="str">
+        <x:v>已采购、品牌型号、位置、安装形式、功率、插头插座、回路、给排水、尺寸或接口中心</x:v>
+      </x:c>
+      <x:c r="N183" t="str">
+        <x:v>confirmed_owner_input_identity_only</x:v>
+      </x:c>
+      <x:c r="O183" t="str">
+        <x:v>1.00</x:v>
+      </x:c>
+      <x:c r="P183" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="Q183" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="R183" t="str"/>
+      <x:c r="S183" t="str"/>
+      <x:c r="T183" t="str">
+        <x:v>2026-08-15</x:v>
+      </x:c>
+      <x:c r="U183" t="str">
+        <x:v>2026-08-15</x:v>
+      </x:c>
+      <x:c r="V183" t="str"/>
+      <x:c r="W183" t="str"/>
+      <x:c r="X183" t="str">
+        <x:v>只登记设备类别与数量；所有安装参数保持 unknown。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:X1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R66fbc29859dd45a1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34695669162a424f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>